<commit_message>
Excel-Export Woche 2 nach dm-Bon aktualisieren
</commit_message>
<xml_diff>
--- a/exports/Urlaubskasse_Woche2.xlsx
+++ b/exports/Urlaubskasse_Woche2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Übersicht" sheetId="1" r:id="R1dec432258d64e0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vorgänge" sheetId="2" r:id="R7f6d3dc429c7480b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kostenblöcke" sheetId="3" r:id="R44574feb646a4ecb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Positionen" sheetId="4" r:id="Rbf4b95d94e5a4462"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Übersicht" sheetId="1" r:id="R3e54fb192e1e4225"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vorgänge" sheetId="2" r:id="R6dfdcfe26b884174"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kostenblöcke" sheetId="3" r:id="Raa8604e2d63d4817"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Positionen" sheetId="4" r:id="R9378c42d0ef44015"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -157,7 +157,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="VorgaengeWoche2" displayName="VorgaengeWoche2" ref="A1:J2" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="VorgaengeWoche2" displayName="VorgaengeWoche2" ref="A1:J4" headerRowCount="1">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Kaufdatum"/>
@@ -175,7 +175,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="KostenbloeckeWoche2" displayName="KostenbloeckeWoche2" ref="A1:F3" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="KostenbloeckeWoche2" displayName="KostenbloeckeWoche2" ref="A1:F6" headerRowCount="1">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Kostenblock"/>
     <x:tableColumn id="2" name="Betrag"/>
@@ -189,7 +189,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="PositionenWoche2" displayName="PositionenWoche2" ref="A1:G59" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="PositionenWoche2" displayName="PositionenWoche2" ref="A1:G106" headerRowCount="1">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Pos."/>
     <x:tableColumn id="2" name="Artikel"/>
@@ -383,7 +383,7 @@
         <x:v>Stand</x:v>
       </x:c>
       <x:c r="B3" s="37" t="str">
-        <x:v>27.07.2026, 12:58 Uhr</x:v>
+        <x:v>27.07.2026, 13:45 Uhr</x:v>
       </x:c>
       <x:c r="C3" s="32"/>
       <x:c r="D3" s="32"/>
@@ -395,7 +395,7 @@
         <x:v>Erfasste Vorgänge</x:v>
       </x:c>
       <x:c r="B4" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C4" s="32"/>
       <x:c r="D4" s="32"/>
@@ -407,7 +407,7 @@
         <x:v>Beleg-/Ausgabensumme</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
-        <x:v>87.79</x:v>
+        <x:v>205.1</x:v>
       </x:c>
       <x:c r="C5" s="32"/>
       <x:c r="D5" s="32"/>
@@ -419,7 +419,7 @@
         <x:v>Ausgeschlossen</x:v>
       </x:c>
       <x:c r="B6" s="16" t="n">
-        <x:v>0</x:v>
+        <x:v>12.05</x:v>
       </x:c>
       <x:c r="C6" s="32"/>
       <x:c r="D6" s="32"/>
@@ -455,14 +455,14 @@
         <x:v>Simon</x:v>
       </x:c>
       <x:c r="B9" s="16" t="n">
-        <x:v>18.93</x:v>
+        <x:v>45.68</x:v>
       </x:c>
       <x:c r="C9" s="16" t="n">
-        <x:v>87.79</x:v>
+        <x:v>188.13</x:v>
       </x:c>
       <x:c r="D9" s="16" t="n">
         <x:f>C9-B9</x:f>
-        <x:v>68.86000000000001</x:v>
+        <x:v>142.45</x:v>
       </x:c>
       <x:c r="E9" s="32"/>
       <x:c r="F9" s="32"/>
@@ -472,14 +472,14 @@
         <x:v>Katrin</x:v>
       </x:c>
       <x:c r="B10" s="16" t="n">
-        <x:v>18.93</x:v>
+        <x:v>45.66</x:v>
       </x:c>
       <x:c r="C10" s="16" t="n">
-        <x:v>0</x:v>
+        <x:v>4.92</x:v>
       </x:c>
       <x:c r="D10" s="16" t="n">
         <x:f>C10-B10</x:f>
-        <x:v>-18.93</x:v>
+        <x:v>-40.739999999999995</x:v>
       </x:c>
       <x:c r="E10" s="32"/>
       <x:c r="F10" s="32"/>
@@ -489,14 +489,14 @@
         <x:v>Hummel W</x:v>
       </x:c>
       <x:c r="B11" s="16" t="n">
-        <x:v>18.93</x:v>
+        <x:v>44.82</x:v>
       </x:c>
       <x:c r="C11" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D11" s="16" t="n">
         <x:f>C11-B11</x:f>
-        <x:v>-18.93</x:v>
+        <x:v>-44.82</x:v>
       </x:c>
       <x:c r="E11" s="32"/>
       <x:c r="F11" s="32"/>
@@ -506,14 +506,14 @@
         <x:v>Hummel M</x:v>
       </x:c>
       <x:c r="B12" s="16" t="n">
-        <x:v>31</x:v>
+        <x:v>56.89</x:v>
       </x:c>
       <x:c r="C12" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D12" s="16" t="n">
         <x:f>C12-B12</x:f>
-        <x:v>-31</x:v>
+        <x:v>-56.89</x:v>
       </x:c>
       <x:c r="E12" s="32"/>
       <x:c r="F12" s="32"/>
@@ -548,7 +548,7 @@
         <x:v>Simon</x:v>
       </x:c>
       <x:c r="C15" s="16" t="n">
-        <x:v>18.93</x:v>
+        <x:v>40.74</x:v>
       </x:c>
       <x:c r="D15" s="32"/>
       <x:c r="E15" s="32"/>
@@ -562,7 +562,7 @@
         <x:v>Simon</x:v>
       </x:c>
       <x:c r="C16" s="16" t="n">
-        <x:v>18.93</x:v>
+        <x:v>44.82</x:v>
       </x:c>
       <x:c r="D16" s="32"/>
       <x:c r="E16" s="32"/>
@@ -576,7 +576,7 @@
         <x:v>Simon</x:v>
       </x:c>
       <x:c r="C17" s="16" t="n">
-        <x:v>31</x:v>
+        <x:v>56.89</x:v>
       </x:c>
       <x:c r="D17" s="32"/>
       <x:c r="E17" s="32"/>
@@ -592,7 +592,7 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="30" t="str">
-        <x:v>Sonderblock: Pueblo Classic sowie Mönchshof Radler, Freiberger Grapefruit, Mönchshof Radler alkoholfrei und Lübzer Zitrone alkoholfrei - jeweils mit Pfand - werden ausschließlich Hummel M zugerechnet.</x:v>
+        <x:v>Sonderblöcke: EDEKA – Pueblo Classic und vier 0,5-l-Getränke inkl. Pfand nur Hummel M. REWE – Laugenstange und Pirulo nur Haushalt Simon &amp; Katrin. dm – nur 3x Barista Hafer, Pinienkerne und Spirelli berücksichtigt.</x:v>
       </x:c>
       <x:c r="B19" s="30"/>
       <x:c r="C19" s="30"/>
@@ -624,13 +624,13 @@
     <x:col min="1" max="1" width="15.25" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="15.880000114440918" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="13.75" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="10.380000114440918" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="9" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="12.5" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="9.380000114440918" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="5.25" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="42" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="44" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -697,10 +697,212 @@
         <x:v>Pueblo + vier 0,5-l-Getränke inkl. Pfand nur Hummel M; Rest je 25 %</x:v>
       </x:c>
     </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>BON-20260725-001</x:v>
+      </x:c>
+      <x:c r="B3" t="n">
+        <x:v>46228.45988425926</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>REWE Markt Christian Schulz oHG</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>Straße am Bahnhof 7, 14547 Beelitz OT Beelitz-Heilstätten</x:v>
+      </x:c>
+      <x:c r="E3" t="n">
+        <x:v>95.41</x:v>
+      </x:c>
+      <x:c r="F3" t="n">
+        <x:v>95.41</x:v>
+      </x:c>
+      <x:c r="G3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H3" t="str">
+        <x:v>Simon</x:v>
+      </x:c>
+      <x:c r="I3" t="str">
+        <x:v>aktiv</x:v>
+      </x:c>
+      <x:c r="J3" t="str">
+        <x:v>Laugenstange + Pirulo nur Haushalt Simon &amp; Katrin; Rest je 25 %</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>BON-20260725-002</x:v>
+      </x:c>
+      <x:c r="B4" t="n">
+        <x:v>46228.4753587963</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>dm-drogerie markt</x:v>
+      </x:c>
+      <x:c r="D4" t="str"/>
+      <x:c r="E4" t="n">
+        <x:v>21.9</x:v>
+      </x:c>
+      <x:c r="F4" t="n">
+        <x:v>9.85</x:v>
+      </x:c>
+      <x:c r="G4" t="n">
+        <x:v>12.05</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>Gemeinschaftskonto Katrin &amp; Simon</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>aktiv</x:v>
+      </x:c>
+      <x:c r="J4" t="str">
+        <x:v>Nur 3x Barista Hafer, Pinienkerne und Spirelli berücksichtigt</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra189dd27dada4673"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85459eaf043c40fd"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="44" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="6.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="6.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="6.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="9.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="9.130000114440918" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="22" t="str">
+        <x:v>Kostenblock</x:v>
+      </x:c>
+      <x:c r="B1" s="22" t="str">
+        <x:v>Betrag</x:v>
+      </x:c>
+      <x:c r="C1" s="22" t="str">
+        <x:v>Simon</x:v>
+      </x:c>
+      <x:c r="D1" s="22" t="str">
+        <x:v>Katrin</x:v>
+      </x:c>
+      <x:c r="E1" s="22" t="str">
+        <x:v>Hummel W</x:v>
+      </x:c>
+      <x:c r="F1" s="22" t="str">
+        <x:v>Hummel M</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="28" t="str">
+        <x:v>Restliche Ausgaben für alle</x:v>
+      </x:c>
+      <x:c r="B2" s="34" t="n">
+        <x:v>75.72</x:v>
+      </x:c>
+      <x:c r="C2" s="34" t="n">
+        <x:v>18.93</x:v>
+      </x:c>
+      <x:c r="D2" s="34" t="n">
+        <x:v>18.93</x:v>
+      </x:c>
+      <x:c r="E2" s="34" t="n">
+        <x:v>18.93</x:v>
+      </x:c>
+      <x:c r="F2" s="34" t="n">
+        <x:v>18.93</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="28" t="str">
+        <x:v>Pueblo + vier 0,5-l-Getränke inkl. Pfand</x:v>
+      </x:c>
+      <x:c r="B3" s="34" t="n">
+        <x:v>12.07</x:v>
+      </x:c>
+      <x:c r="C3" s="34" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D3" s="34" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E3" s="34" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F3" s="34" t="n">
+        <x:v>12.07</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>REWE: Restliche Ausgaben für alle</x:v>
+      </x:c>
+      <x:c r="B4" t="n">
+        <x:v>93.72</x:v>
+      </x:c>
+      <x:c r="C4" t="n">
+        <x:v>23.43</x:v>
+      </x:c>
+      <x:c r="D4" t="n">
+        <x:v>23.43</x:v>
+      </x:c>
+      <x:c r="E4" t="n">
+        <x:v>23.43</x:v>
+      </x:c>
+      <x:c r="F4" t="n">
+        <x:v>23.43</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>REWE: Laugenstange + Pirulo, Haushalt Simon &amp; Katrin</x:v>
+      </x:c>
+      <x:c r="B5" t="n">
+        <x:v>1.69</x:v>
+      </x:c>
+      <x:c r="C5" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="D5" t="n">
+        <x:v>0.84</x:v>
+      </x:c>
+      <x:c r="E5" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F5" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>dm: 3x Barista Hafer, Pinienkerne und Spirelli</x:v>
+      </x:c>
+      <x:c r="B6" t="n">
+        <x:v>9.85</x:v>
+      </x:c>
+      <x:c r="C6" t="n">
+        <x:v>2.47</x:v>
+      </x:c>
+      <x:c r="D6" t="n">
+        <x:v>2.46</x:v>
+      </x:c>
+      <x:c r="E6" t="n">
+        <x:v>2.46</x:v>
+      </x:c>
+      <x:c r="F6" t="n">
+        <x:v>2.46</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04ef55592f924608"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -715,7 +917,7 @@
     <x:col min="4" max="4" width="7.880000114440918" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="8.630000114440918" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="5.75" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="25" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -1971,10 +2173,1027 @@
         <x:v>Gemeinschaft</x:v>
       </x:c>
     </x:row>
+    <x:row r="60">
+      <x:c r="A60" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B60" t="str">
+        <x:v>Johannisbeere</x:v>
+      </x:c>
+      <x:c r="C60" t="n">
+        <x:v>0.47</x:v>
+      </x:c>
+      <x:c r="D60" t="str">
+        <x:v>kg</x:v>
+      </x:c>
+      <x:c r="E60" t="n">
+        <x:v>5.98</x:v>
+      </x:c>
+      <x:c r="F60" t="n">
+        <x:v>2.81</x:v>
+      </x:c>
+      <x:c r="G60" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B61" t="str">
+        <x:v>Banane Chiquita</x:v>
+      </x:c>
+      <x:c r="C61" t="n">
+        <x:v>0.922</x:v>
+      </x:c>
+      <x:c r="D61" t="str">
+        <x:v>kg</x:v>
+      </x:c>
+      <x:c r="E61" t="n">
+        <x:v>2.49</x:v>
+      </x:c>
+      <x:c r="F61" t="n">
+        <x:v>2.3</x:v>
+      </x:c>
+      <x:c r="G61" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B62" t="str">
+        <x:v>Bio Feta 45 %</x:v>
+      </x:c>
+      <x:c r="C62" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D62" t="str">
+        <x:v>Stk.</x:v>
+      </x:c>
+      <x:c r="E62" t="n">
+        <x:v>2.69</x:v>
+      </x:c>
+      <x:c r="F62" t="n">
+        <x:v>8.07</x:v>
+      </x:c>
+      <x:c r="G62" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B63" t="str">
+        <x:v>Bio Hirtenkäse</x:v>
+      </x:c>
+      <x:c r="C63" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D63" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E63"/>
+      <x:c r="F63" t="n">
+        <x:v>2.19</x:v>
+      </x:c>
+      <x:c r="G63" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B64" t="str">
+        <x:v>Laugenstange</x:v>
+      </x:c>
+      <x:c r="C64" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D64" t="str">
+        <x:v>Stk.</x:v>
+      </x:c>
+      <x:c r="E64"/>
+      <x:c r="F64" t="n">
+        <x:v>0.39</x:v>
+      </x:c>
+      <x:c r="G64" t="str">
+        <x:v>Haushalt Simon &amp; Katrin</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B65" t="str">
+        <x:v>Zitrone Bio</x:v>
+      </x:c>
+      <x:c r="C65" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D65" t="str">
+        <x:v>Stk.</x:v>
+      </x:c>
+      <x:c r="E65" t="n">
+        <x:v>2.29</x:v>
+      </x:c>
+      <x:c r="F65" t="n">
+        <x:v>9.16</x:v>
+      </x:c>
+      <x:c r="G65" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B66" t="str">
+        <x:v>Erdbeere Premium</x:v>
+      </x:c>
+      <x:c r="C66" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D66" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E66"/>
+      <x:c r="F66" t="n">
+        <x:v>2.49</x:v>
+      </x:c>
+      <x:c r="G66" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B67" t="str">
+        <x:v>Apfelchips Bio</x:v>
+      </x:c>
+      <x:c r="C67" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D67" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E67"/>
+      <x:c r="F67" t="n">
+        <x:v>2.49</x:v>
+      </x:c>
+      <x:c r="G67" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B68" t="str">
+        <x:v>Kiwi Bio</x:v>
+      </x:c>
+      <x:c r="C68" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D68" t="str">
+        <x:v>Stk.</x:v>
+      </x:c>
+      <x:c r="E68" t="n">
+        <x:v>0.79</x:v>
+      </x:c>
+      <x:c r="F68" t="n">
+        <x:v>2.37</x:v>
+      </x:c>
+      <x:c r="G68" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B69" t="str">
+        <x:v>Schalotten Bio</x:v>
+      </x:c>
+      <x:c r="C69" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D69" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E69"/>
+      <x:c r="F69" t="n">
+        <x:v>1.69</x:v>
+      </x:c>
+      <x:c r="G69" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B70" t="str">
+        <x:v>Cherry Rispe Bio</x:v>
+      </x:c>
+      <x:c r="C70" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D70" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E70" t="n">
+        <x:v>3.29</x:v>
+      </x:c>
+      <x:c r="F70" t="n">
+        <x:v>6.58</x:v>
+      </x:c>
+      <x:c r="G70" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B71" t="str">
+        <x:v>Tomate Bio</x:v>
+      </x:c>
+      <x:c r="C71" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D71" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E71" t="n">
+        <x:v>2.19</x:v>
+      </x:c>
+      <x:c r="F71" t="n">
+        <x:v>6.57</x:v>
+      </x:c>
+      <x:c r="G71" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B72" t="str">
+        <x:v>Zucchini Bio</x:v>
+      </x:c>
+      <x:c r="C72" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D72" t="str">
+        <x:v>Stk.</x:v>
+      </x:c>
+      <x:c r="E72" t="n">
+        <x:v>1.11</x:v>
+      </x:c>
+      <x:c r="F72" t="n">
+        <x:v>2.22</x:v>
+      </x:c>
+      <x:c r="G72" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B73" t="str">
+        <x:v>Champignons braun Bio</x:v>
+      </x:c>
+      <x:c r="C73" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D73" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E73" t="n">
+        <x:v>1.99</x:v>
+      </x:c>
+      <x:c r="F73" t="n">
+        <x:v>7.96</x:v>
+      </x:c>
+      <x:c r="G73" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B74" t="str">
+        <x:v>Petersilie</x:v>
+      </x:c>
+      <x:c r="C74" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D74" t="str">
+        <x:v>Bund</x:v>
+      </x:c>
+      <x:c r="E74"/>
+      <x:c r="F74" t="n">
+        <x:v>1.69</x:v>
+      </x:c>
+      <x:c r="G74" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B75" t="str">
+        <x:v>Bio Eier OKT</x:v>
+      </x:c>
+      <x:c r="C75" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D75" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E75"/>
+      <x:c r="F75" t="n">
+        <x:v>3.99</x:v>
+      </x:c>
+      <x:c r="G75" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B76" t="str">
+        <x:v>Bio Fassbutter Sauerrahm</x:v>
+      </x:c>
+      <x:c r="C76" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D76" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E76"/>
+      <x:c r="F76" t="n">
+        <x:v>4.49</x:v>
+      </x:c>
+      <x:c r="G76" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B77" t="str">
+        <x:v>Bio Crème fraîche</x:v>
+      </x:c>
+      <x:c r="C77" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D77" t="str">
+        <x:v>Becher</x:v>
+      </x:c>
+      <x:c r="E77"/>
+      <x:c r="F77" t="n">
+        <x:v>1.09</x:v>
+      </x:c>
+      <x:c r="G77" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B78" t="str">
+        <x:v>Bio Joghurt 3,8 %</x:v>
+      </x:c>
+      <x:c r="C78" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D78" t="str">
+        <x:v>Becher</x:v>
+      </x:c>
+      <x:c r="E78" t="n">
+        <x:v>1.15</x:v>
+      </x:c>
+      <x:c r="F78" t="n">
+        <x:v>2.3</x:v>
+      </x:c>
+      <x:c r="G78" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B79" t="str">
+        <x:v>TK Junge Erbsen</x:v>
+      </x:c>
+      <x:c r="C79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D79" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E79"/>
+      <x:c r="F79" t="n">
+        <x:v>1.89</x:v>
+      </x:c>
+      <x:c r="G79" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B80" t="str">
+        <x:v>Bio TK Himbeeren</x:v>
+      </x:c>
+      <x:c r="C80" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D80" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E80"/>
+      <x:c r="F80" t="n">
+        <x:v>3.79</x:v>
+      </x:c>
+      <x:c r="G80" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B81" t="str">
+        <x:v>Pirulo Watermelo</x:v>
+      </x:c>
+      <x:c r="C81" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D81" t="str">
+        <x:v>Stk.</x:v>
+      </x:c>
+      <x:c r="E81"/>
+      <x:c r="F81" t="n">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="G81" t="str">
+        <x:v>Haushalt Simon &amp; Katrin</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B82" t="str">
+        <x:v>Kritharaki</x:v>
+      </x:c>
+      <x:c r="C82" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D82" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E82" t="n">
+        <x:v>1.69</x:v>
+      </x:c>
+      <x:c r="F82" t="n">
+        <x:v>3.38</x:v>
+      </x:c>
+      <x:c r="G82" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B83" t="str">
+        <x:v>Apfelmark</x:v>
+      </x:c>
+      <x:c r="C83" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D83" t="str">
+        <x:v>Glas</x:v>
+      </x:c>
+      <x:c r="E83"/>
+      <x:c r="F83" t="n">
+        <x:v>1.49</x:v>
+      </x:c>
+      <x:c r="G83" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B84" t="str">
+        <x:v>Spreelinge</x:v>
+      </x:c>
+      <x:c r="C84" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D84" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E84"/>
+      <x:c r="F84" t="n">
+        <x:v>2.59</x:v>
+      </x:c>
+      <x:c r="G84" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B85" t="str">
+        <x:v>Riffelchips Salz</x:v>
+      </x:c>
+      <x:c r="C85" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D85" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E85" t="n">
+        <x:v>1.39</x:v>
+      </x:c>
+      <x:c r="F85" t="n">
+        <x:v>2.78</x:v>
+      </x:c>
+      <x:c r="G85" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B86" t="str">
+        <x:v>Honig-Salz-Mandeln</x:v>
+      </x:c>
+      <x:c r="C86" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D86" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E86"/>
+      <x:c r="F86" t="n">
+        <x:v>1.69</x:v>
+      </x:c>
+      <x:c r="G86" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B87" t="str">
+        <x:v>Grün-Ohr Hase</x:v>
+      </x:c>
+      <x:c r="C87" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D87" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E87"/>
+      <x:c r="F87" t="n">
+        <x:v>0.77</x:v>
+      </x:c>
+      <x:c r="G87" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B88" t="str">
+        <x:v>Fred Ferkel</x:v>
+      </x:c>
+      <x:c r="C88" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D88" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E88"/>
+      <x:c r="F88" t="n">
+        <x:v>0.77</x:v>
+      </x:c>
+      <x:c r="G88" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B89" t="str">
+        <x:v>Katjes Wunderland</x:v>
+      </x:c>
+      <x:c r="C89" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D89" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E89"/>
+      <x:c r="F89" t="n">
+        <x:v>0.77</x:v>
+      </x:c>
+      <x:c r="G89" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B90" t="str">
+        <x:v>Cola Life Sour</x:v>
+      </x:c>
+      <x:c r="C90" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D90" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E90"/>
+      <x:c r="F90" t="n">
+        <x:v>0.77</x:v>
+      </x:c>
+      <x:c r="G90" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B91" t="str">
+        <x:v>Mineralwasser Glas</x:v>
+      </x:c>
+      <x:c r="C91" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D91" t="str">
+        <x:v>Flasche</x:v>
+      </x:c>
+      <x:c r="E91" t="n">
+        <x:v>0.89</x:v>
+      </x:c>
+      <x:c r="F91" t="n">
+        <x:v>2.67</x:v>
+      </x:c>
+      <x:c r="G91" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B92" t="str">
+        <x:v>Pfand Mineralwasser Glas</x:v>
+      </x:c>
+      <x:c r="C92" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D92" t="str">
+        <x:v>Pfand</x:v>
+      </x:c>
+      <x:c r="E92" t="n">
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="F92" t="n">
+        <x:v>0.45</x:v>
+      </x:c>
+      <x:c r="G92" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B93" t="str">
+        <x:v>Leergut Mehrweg</x:v>
+      </x:c>
+      <x:c r="C93" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D93" t="str">
+        <x:v>Gutschrift</x:v>
+      </x:c>
+      <x:c r="E93"/>
+      <x:c r="F93" t="n">
+        <x:v>-0.15</x:v>
+      </x:c>
+      <x:c r="G93" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B94" t="str">
+        <x:v>Leergut Mehrweg</x:v>
+      </x:c>
+      <x:c r="C94" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D94" t="str">
+        <x:v>Gutschrift</x:v>
+      </x:c>
+      <x:c r="E94"/>
+      <x:c r="F94" t="n">
+        <x:v>-0.15</x:v>
+      </x:c>
+      <x:c r="G94" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B95" t="str">
+        <x:v>Leergut Einweg</x:v>
+      </x:c>
+      <x:c r="C95" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D95" t="str">
+        <x:v>Gutschrift</x:v>
+      </x:c>
+      <x:c r="E95"/>
+      <x:c r="F95" t="n">
+        <x:v>-0.25</x:v>
+      </x:c>
+      <x:c r="G95" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B96" t="str">
+        <x:v>Sanft &amp; Sicher DP 2x50 St</x:v>
+      </x:c>
+      <x:c r="C96" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D96" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E96"/>
+      <x:c r="F96" t="n">
+        <x:v>2.95</x:v>
+      </x:c>
+      <x:c r="G96" t="str">
+        <x:v>Ausgeschlossen</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B97" t="str">
+        <x:v>dmBio Barista Hafer Drink</x:v>
+      </x:c>
+      <x:c r="C97" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D97" t="str">
+        <x:v>Stk.</x:v>
+      </x:c>
+      <x:c r="E97" t="n">
+        <x:v>1.35</x:v>
+      </x:c>
+      <x:c r="F97" t="n">
+        <x:v>4.05</x:v>
+      </x:c>
+      <x:c r="G97" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B98" t="str">
+        <x:v>dmBio Mandeln 200 g</x:v>
+      </x:c>
+      <x:c r="C98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D98" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E98"/>
+      <x:c r="F98" t="n">
+        <x:v>2.55</x:v>
+      </x:c>
+      <x:c r="G98" t="str">
+        <x:v>Ausgeschlossen</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B99" t="str">
+        <x:v>dmBio Pinienkerne 60 g</x:v>
+      </x:c>
+      <x:c r="C99" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D99" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E99"/>
+      <x:c r="F99" t="n">
+        <x:v>4.95</x:v>
+      </x:c>
+      <x:c r="G99" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B100" t="str">
+        <x:v>dmBio Hanfsamen geschält 200 g</x:v>
+      </x:c>
+      <x:c r="C100" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D100" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E100"/>
+      <x:c r="F100" t="n">
+        <x:v>2.95</x:v>
+      </x:c>
+      <x:c r="G100" t="str">
+        <x:v>Ausgeschlossen</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101">
+      <x:c r="A101" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B101" t="str">
+        <x:v>dmBio Leinsamen ganz 500 g</x:v>
+      </x:c>
+      <x:c r="C101" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D101" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E101"/>
+      <x:c r="F101" t="n">
+        <x:v>1.55</x:v>
+      </x:c>
+      <x:c r="G101" t="str">
+        <x:v>Ausgeschlossen</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102">
+      <x:c r="A102" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B102" t="str">
+        <x:v>dmBio Spirelli 500 g</x:v>
+      </x:c>
+      <x:c r="C102" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D102" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E102"/>
+      <x:c r="F102" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="G102" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103">
+      <x:c r="A103" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B103" t="str">
+        <x:v>dmBio Gemüsebrühwürfel 66 g</x:v>
+      </x:c>
+      <x:c r="C103" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D103" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E103"/>
+      <x:c r="F103" t="n">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="G103" t="str">
+        <x:v>Ausgeschlossen</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104">
+      <x:c r="A104" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B104" t="str">
+        <x:v>Coupon dmBio Gemüsebrühwürfel</x:v>
+      </x:c>
+      <x:c r="C104" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D104" t="str">
+        <x:v>Coupon</x:v>
+      </x:c>
+      <x:c r="E104"/>
+      <x:c r="F104" t="n">
+        <x:v>-0.75</x:v>
+      </x:c>
+      <x:c r="G104" t="str">
+        <x:v>Ausgeschlossen</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105">
+      <x:c r="A105" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B105" t="str">
+        <x:v>dmBio Haferflocken Feinblatt 1000 g</x:v>
+      </x:c>
+      <x:c r="C105" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D105" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E105"/>
+      <x:c r="F105" t="n">
+        <x:v>1.55</x:v>
+      </x:c>
+      <x:c r="G105" t="str">
+        <x:v>Ausgeschlossen</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106">
+      <x:c r="A106" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B106" t="str">
+        <x:v>Mivolis Vitamin C Brausetabletten</x:v>
+      </x:c>
+      <x:c r="C106" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D106" t="str">
+        <x:v>Packung</x:v>
+      </x:c>
+      <x:c r="E106"/>
+      <x:c r="F106" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="G106" t="str">
+        <x:v>Ausgeschlossen</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8bae2b78713942db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e2fa4ed642342a1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>